<commit_message>
Mere fra Jan Brown Consulting session
</commit_message>
<xml_diff>
--- a/modeller/Use Case.xlsx
+++ b/modeller/Use Case.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Datamatiker\Projekter\Hydac\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frede\git\HYDAC\Modeller\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB5BB8D8-FF5E-4456-B0A0-90F19AFBD58E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0DA9E23-82E8-4289-84FF-324E25760103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="561" xr2:uid="{FAE73960-6D5B-49EE-8D5E-7E75CD0D9398}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="52">
   <si>
     <t>Primær aktør</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Medarbejder</t>
   </si>
   <si>
-    <t>1. Medarbejder møder ind om morgnen</t>
-  </si>
-  <si>
     <t>2. Medarbejder går hen til skærmen</t>
   </si>
   <si>
@@ -80,30 +77,12 @@
     <t>5. Medarbejder trykker "Ankomst"</t>
   </si>
   <si>
-    <t>6. Medarbejder vælger smiley efter humør, rød gul grøn, eller blank</t>
-  </si>
-  <si>
-    <t>7. System melder "God dag"</t>
-  </si>
-  <si>
     <t>UC2</t>
   </si>
   <si>
     <t>1. Medarbejder går hen til skærmen</t>
   </si>
   <si>
-    <t>8. Medarbejderens dag er slut</t>
-  </si>
-  <si>
-    <t>Gentage trin 2-4</t>
-  </si>
-  <si>
-    <t>9. Medarbejder trykker "Afgang"</t>
-  </si>
-  <si>
-    <t>10. Systemet skriver "God dag" og timerne bliver registreret til lønafdelingen</t>
-  </si>
-  <si>
     <t>Medarbejder booker møde med kunde</t>
   </si>
   <si>
@@ -146,15 +125,6 @@
     <t xml:space="preserve">Medarbejder </t>
   </si>
   <si>
-    <t>Tjek ind og ud</t>
-  </si>
-  <si>
-    <t>Tjekker ind om morgenen, og ud efter arbejde</t>
-  </si>
-  <si>
-    <t>Registrere sin ankomst, og melde sin afgang</t>
-  </si>
-  <si>
     <t>Besøgende</t>
   </si>
   <si>
@@ -186,6 +156,45 @@
   </si>
   <si>
     <t>8. Systemet giver reception? Besked, og ansvarlige for møde bliver advaret.</t>
+  </si>
+  <si>
+    <t>Tjekker ud efter arbejde</t>
+  </si>
+  <si>
+    <t>Tjek ud</t>
+  </si>
+  <si>
+    <t>UC4</t>
+  </si>
+  <si>
+    <t>Melder sin afgang</t>
+  </si>
+  <si>
+    <t>1. Medarbejderens dag er slut.</t>
+  </si>
+  <si>
+    <t>5. Medarbejder trykker "Afgang"</t>
+  </si>
+  <si>
+    <t>6. System melder "God dag"</t>
+  </si>
+  <si>
+    <t>Tjekker ind om morgenen</t>
+  </si>
+  <si>
+    <t>1. Medarbejder møder ind om morgenen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tjek ind </t>
+  </si>
+  <si>
+    <t>Registrere sin ankomst</t>
+  </si>
+  <si>
+    <t>6. Medarbejder vælger smiley efter humør, rød, gul, grøn, eller blank</t>
+  </si>
+  <si>
+    <t>7. System melder "*Ankomst registreret*"</t>
   </si>
 </sst>
 </file>
@@ -221,7 +230,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -229,18 +238,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -575,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39673B22-004F-4717-8A37-72698BEC2F7D}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.265625" bestFit="1" customWidth="1"/>
@@ -584,263 +624,328 @@
     <col min="5" max="5" width="63.73046875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.265625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="63.73046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="54.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="D1" s="1" t="s">
+      <c r="B1" s="3"/>
+      <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1"/>
-      <c r="G1" s="1" t="s">
+      <c r="E1" s="3"/>
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
+      <c r="H1" s="3"/>
+      <c r="J1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="3"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="3" t="s">
+      <c r="G5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="1"/>
+      <c r="H8" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="J8" s="1"/>
+      <c r="K8" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="1"/>
+      <c r="H9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J9" s="1"/>
+      <c r="K9" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A10" s="1"/>
+      <c r="B10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="1"/>
+      <c r="H10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10" s="1"/>
+      <c r="K10" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A11" s="1"/>
+      <c r="B11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="1"/>
+      <c r="H11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="H4" s="3" t="s">
+      <c r="J11" s="1"/>
+      <c r="K11" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A12" s="1"/>
+      <c r="B12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="1"/>
+      <c r="H12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J12" s="1"/>
+      <c r="K12" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A13" s="1"/>
+      <c r="B13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" s="1"/>
+      <c r="H13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J13" s="1"/>
+      <c r="K13" s="2"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A14" s="1"/>
+      <c r="B14" s="2"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="1"/>
+      <c r="H14" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A5" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" s="2"/>
-      <c r="H9" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A12" s="2"/>
-      <c r="B12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A14" s="4"/>
-      <c r="B14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G14" s="4"/>
-      <c r="H14" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A15" s="4"/>
-      <c r="B15" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A16" s="4"/>
-      <c r="B16" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A17" s="4"/>
-      <c r="B17" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="J14" s="1"/>
+      <c r="K14" s="2"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A15" s="1"/>
+      <c r="B15" s="2"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="2"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A16" s="1"/>
+      <c r="B16" s="2"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="2"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A17" s="1"/>
+      <c r="B17" s="2"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="G1:H1"/>
+    <mergeCell ref="J1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>